<commit_message>
Add 2025 Grade 3 high-school mock exam for 구성관 class and 2025 middle-1 exams for 이서연 class
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bh4sYU41PMoBKwVo8YRab
</commit_message>
<xml_diff>
--- a/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
+++ b/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
@@ -12,6 +12,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="고1 모의고사" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="고2 모의고사" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="고3 모의고사_수능" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="56">
   <si>
     <r>
       <rPr>
@@ -575,6 +576,144 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모의고사</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3(2025) 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">듣기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">독해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">총점 표와 그래프</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">읽는 법</t>
   </si>
   <si>
@@ -813,24 +952,24 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· 2025</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">년 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3·4</t>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 4</t>
     </r>
     <r>
       <rPr>
@@ -855,24 +994,154 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">모의고사는 받은 사진에 기록이 없어 고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시트가 없습니다</t>
+      <t xml:space="preserve">모의고사는 성적표에 아직 기록이 없습니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 구성관 총점은 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2025</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">년 성적표 두 장에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">92</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">점과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">93</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">점으로 다르게 적혀 있어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">듣기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">독해 개수가 함께 적힌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">92</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">점을 사용했습니다</t>
     </r>
     <r>
       <rPr>
@@ -1156,6 +1425,55 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">모의고사</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모의고사</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수능</t>
     </r>
   </si>
   <si>
@@ -2341,6 +2659,287 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모의고사</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">구성관 반 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">고</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모의고사</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수능 성적 변화</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3(2025) 3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">· </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">파란 글씨 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">성적표 입력값</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검은 글씨 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계산식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">빈칸 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">기록 없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF666666"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">미응시</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">중</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 3</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차
+고</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
     </r>
     <r>
       <rPr>
@@ -3247,11 +3846,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="82110438"/>
-        <c:axId val="8631828"/>
+        <c:axId val="83324924"/>
+        <c:axId val="4556809"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="82110438"/>
+        <c:axId val="83324924"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3283,7 +3882,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8631828"/>
+        <c:crossAx val="4556809"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3291,7 +3890,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="8631828"/>
+        <c:axId val="4556809"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -3369,7 +3968,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82110438"/>
+        <c:crossAx val="83324924"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -3982,11 +4581,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="90790734"/>
-        <c:axId val="67619163"/>
+        <c:axId val="50954600"/>
+        <c:axId val="73400679"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="90790734"/>
+        <c:axId val="50954600"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4018,7 +4617,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67619163"/>
+        <c:crossAx val="73400679"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4026,7 +4625,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67619163"/>
+        <c:axId val="73400679"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -4104,7 +4703,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90790734"/>
+        <c:crossAx val="50954600"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -4717,11 +5316,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="10321976"/>
-        <c:axId val="65756103"/>
+        <c:axId val="2433333"/>
+        <c:axId val="27384686"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10321976"/>
+        <c:axId val="2433333"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4753,7 +5352,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65756103"/>
+        <c:crossAx val="27384686"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4761,7 +5360,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="65756103"/>
+        <c:axId val="27384686"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -4839,7 +5438,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10321976"/>
+        <c:crossAx val="2433333"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -5368,11 +5967,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="69235447"/>
-        <c:axId val="39588961"/>
+        <c:axId val="53738799"/>
+        <c:axId val="77088438"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="69235447"/>
+        <c:axId val="53738799"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5404,7 +6003,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="39588961"/>
+        <c:crossAx val="77088438"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5412,7 +6011,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="39588961"/>
+        <c:axId val="77088438"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -5490,7 +6089,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69235447"/>
+        <c:crossAx val="53738799"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -6019,11 +6618,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="87152608"/>
-        <c:axId val="29627265"/>
+        <c:axId val="17587937"/>
+        <c:axId val="52720770"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87152608"/>
+        <c:axId val="17587937"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6055,7 +6654,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29627265"/>
+        <c:crossAx val="52720770"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6063,7 +6662,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29627265"/>
+        <c:axId val="52720770"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -6141,7 +6740,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87152608"/>
+        <c:crossAx val="17587937"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -6670,11 +7269,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="30776371"/>
-        <c:axId val="69179502"/>
+        <c:axId val="73983087"/>
+        <c:axId val="94289784"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="30776371"/>
+        <c:axId val="73983087"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6706,7 +7305,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69179502"/>
+        <c:crossAx val="94289784"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6714,7 +7313,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69179502"/>
+        <c:axId val="94289784"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -6792,7 +7391,1708 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30776371"/>
+        <c:crossAx val="73983087"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="2"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>고3 모의고사·수능 · 총점</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A6</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>구성관</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4a7ebb"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A7</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>송지효</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="be4b48"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A8</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>신준섭</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="98b855"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>87</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>박주연</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7d5fa0"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>82</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:axId val="84048133"/>
+        <c:axId val="52934726"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="84048133"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="52934726"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="52934726"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="100"/>
+          <c:min val="40"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>점 / 100</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="84048133"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="10"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>고3 모의고사·수능 · 듣기</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>구성관</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4a7ebb"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A15</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>송지효</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="be4b48"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$15</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A16</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>신준섭</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="98b855"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A17</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>박주연</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7d5fa0"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>17</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:axId val="16593772"/>
+        <c:axId val="48756552"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="16593772"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="48756552"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="48756552"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="17"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>맞은 개수 / 17</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="16593772"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="1"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>고3 모의고사·수능 · 독해</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A22</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>구성관</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4a7ebb"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4a7ebb"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$22</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A23</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>송지효</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="be4b48"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="be4b48"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>28</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A24</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>신준섭</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="98b855"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="98b855"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$24</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>23</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!A25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>박주연</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7d5fa0"/>
+            </a:solidFill>
+            <a:ln w="28440">
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="7d5fa0"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>중3 3차
+고3 모의고사</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'고3 모의고사_수능'!$B$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>20</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:hiLowLines>
+          <c:spPr>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:hiLowLines>
+        <c:marker val="1"/>
+        <c:axId val="28008604"/>
+        <c:axId val="77983308"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="28008604"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="77983308"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="77983308"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="28"/>
+          <c:min val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>맞은 개수 / 28</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="28008604"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -7035,6 +9335,101 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>134640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>255960</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>72360</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5122440" y="571680"/>
+        <a:ext cx="5759640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>134640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>255960</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>119520</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5122440" y="4095720"/>
+        <a:ext cx="5759640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>134640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>255960</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>167040</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="8" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5122440" y="7381800"/>
+        <a:ext cx="5759640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -7215,7 +9610,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -7254,16 +9649,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A9" s="3"/>
     </row>
-    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -7272,22 +9667,32 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A13" s="3"/>
     </row>
-    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -7306,7 +9711,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -7318,37 +9723,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">'고1 모의고사'!I10</f>
@@ -7365,10 +9770,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">'고1 모의고사'!I18</f>
@@ -7385,10 +9790,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">'고1 모의고사'!I26</f>
@@ -7405,10 +9810,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">'고2 모의고사'!F10</f>
@@ -7425,10 +9830,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>23</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>21</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">'고2 모의고사'!F18</f>
@@ -7445,10 +9850,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">'고2 모의고사'!F26</f>
@@ -7461,6 +9866,66 @@
       <c r="E10" s="9" t="n">
         <f aca="false">D10-C10</f>
         <v>-0.25</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!C10</f>
+        <v>92.25</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!D10</f>
+        <v>92.25</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <f aca="false">D11-C11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!C18</f>
+        <v>17</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!D18</f>
+        <v>17</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <f aca="false">D12-C12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!C26</f>
+        <v>24.75</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <f aca="false">'고3 모의고사_수능'!D26</f>
+        <v>24.75</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <f aca="false">D13-C13</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -7488,57 +9953,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>71</v>
@@ -7576,7 +10041,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>58</v>
@@ -7614,7 +10079,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>70</v>
@@ -7652,7 +10117,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>69</v>
@@ -7690,7 +10155,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
@@ -7735,47 +10200,47 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>17</v>
@@ -7813,7 +10278,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>15</v>
@@ -7851,7 +10316,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>16</v>
@@ -7889,7 +10354,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>17</v>
@@ -7927,7 +10392,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
@@ -7972,47 +10437,47 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B22" s="10" t="n">
         <v>16</v>
@@ -8050,7 +10515,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>12</v>
@@ -8088,7 +10553,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>16</v>
@@ -8126,7 +10591,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>15</v>
@@ -8164,7 +10629,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>
@@ -8233,48 +10698,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>89</v>
@@ -8303,7 +10768,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>92</v>
@@ -8332,7 +10797,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>94</v>
@@ -8361,7 +10826,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>69</v>
@@ -8390,7 +10855,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
@@ -8423,38 +10888,38 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>16</v>
@@ -8483,7 +10948,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>17</v>
@@ -8512,7 +10977,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>17</v>
@@ -8541,7 +11006,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>16</v>
@@ -8570,7 +11035,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
@@ -8603,38 +11068,38 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B22" s="10" t="n">
         <v>25</v>
@@ -8663,7 +11128,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>25</v>
@@ -8692,7 +11157,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>26</v>
@@ -8721,7 +11186,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>17</v>
@@ -8750,7 +11215,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>
@@ -8779,6 +11244,409 @@
       <c r="H26" s="14" t="n">
         <f aca="false">G26-F26</f>
         <v>-0.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <f aca="false">B6</f>
+        <v>100</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B6:B6)</f>
+        <v>100</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <f aca="false">D6-C6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <f aca="false">B7</f>
+        <v>100</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B7:B7)</f>
+        <v>100</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">D7-C7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <f aca="false">B8</f>
+        <v>87</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B8:B8)</f>
+        <v>87</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <f aca="false">D8-C8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <f aca="false">B9</f>
+        <v>82</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B9:B9)</f>
+        <v>82</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <f aca="false">D9-C9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="13" t="n">
+        <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
+        <v>92.25</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <f aca="false">B10</f>
+        <v>92.25</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B10:B10)</f>
+        <v>92.25</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">D10-C10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <f aca="false">B14</f>
+        <v>17</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B14:B14)</f>
+        <v>17</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <f aca="false">D14-C14</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <f aca="false">B15</f>
+        <v>17</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B15:B15)</f>
+        <v>17</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <f aca="false">D15-C15</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <f aca="false">B16</f>
+        <v>17</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B16:B16)</f>
+        <v>17</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <f aca="false">D16-C16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <f aca="false">B17</f>
+        <v>17</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B17:B17)</f>
+        <v>17</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <f aca="false">D17-C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="13" t="n">
+        <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
+        <v>17</v>
+      </c>
+      <c r="C18" s="13" t="n">
+        <f aca="false">B18</f>
+        <v>17</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B18:B18)</f>
+        <v>17</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <f aca="false">D18-C18</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <f aca="false">B22</f>
+        <v>28</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B22:B22)</f>
+        <v>28</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <f aca="false">D22-C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <f aca="false">B23</f>
+        <v>28</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B23:B23)</f>
+        <v>28</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <f aca="false">D23-C23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <f aca="false">B24</f>
+        <v>23</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B24:B24)</f>
+        <v>23</v>
+      </c>
+      <c r="E24" s="11" t="n">
+        <f aca="false">D24-C24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <f aca="false">B25</f>
+        <v>20</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B25:B25)</f>
+        <v>20</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <f aca="false">D25-C25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="13" t="n">
+        <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>
+        <v>24.75</v>
+      </c>
+      <c r="C26" s="13" t="n">
+        <f aca="false">B26</f>
+        <v>24.75</v>
+      </c>
+      <c r="D26" s="13" t="n">
+        <f aca="false">LOOKUP(9.99E+307,B26:B26)</f>
+        <v>24.75</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <f aca="false">D26-C26</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclude 2026 CSAT (4th exam) from 구성관 class comparison and label its group as 고3 모의고사
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bh4sYU41PMoBKwVo8YRab
</commit_message>
<xml_diff>
--- a/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
+++ b/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
@@ -12,7 +12,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="고1 모의고사" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="고2 모의고사" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="고3 모의고사_수능" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="고3 모의고사" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -617,23 +617,6 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수능</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">: </t>
     </r>
     <r>
@@ -977,24 +960,75 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">차 고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">모의고사는 성적표에 아직 기록이 없습니다</t>
+      <t xml:space="preserve">차</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">학년도 수능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 난이도가 매우 높았던 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">불수능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이라 비교에서 제외했습니다</t>
     </r>
     <r>
       <rPr>
@@ -1455,25 +1489,6 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">모의고사</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수능</t>
     </r>
   </si>
   <si>
@@ -2716,26 +2731,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">모의고사</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="14"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">수능 성적 변화</t>
+      <t xml:space="preserve">모의고사 성적 변화</t>
     </r>
   </si>
   <si>
@@ -3846,11 +3842,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="83324924"/>
-        <c:axId val="4556809"/>
+        <c:axId val="16752297"/>
+        <c:axId val="73426723"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="83324924"/>
+        <c:axId val="16752297"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3882,7 +3878,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4556809"/>
+        <c:crossAx val="73426723"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3890,7 +3886,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="4556809"/>
+        <c:axId val="73426723"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -3968,7 +3964,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83324924"/>
+        <c:crossAx val="16752297"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -4581,11 +4577,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="50954600"/>
-        <c:axId val="73400679"/>
+        <c:axId val="10296452"/>
+        <c:axId val="13529544"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="50954600"/>
+        <c:axId val="10296452"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4617,7 +4613,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73400679"/>
+        <c:crossAx val="13529544"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4625,7 +4621,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="73400679"/>
+        <c:axId val="13529544"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -4703,7 +4699,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50954600"/>
+        <c:crossAx val="10296452"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -5316,11 +5312,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="2433333"/>
-        <c:axId val="27384686"/>
+        <c:axId val="38405688"/>
+        <c:axId val="69754615"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2433333"/>
+        <c:axId val="38405688"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5352,7 +5348,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27384686"/>
+        <c:crossAx val="69754615"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5360,7 +5356,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="27384686"/>
+        <c:axId val="69754615"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -5438,7 +5434,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2433333"/>
+        <c:crossAx val="38405688"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -5967,11 +5963,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="53738799"/>
-        <c:axId val="77088438"/>
+        <c:axId val="43587432"/>
+        <c:axId val="46670391"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="53738799"/>
+        <c:axId val="43587432"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6003,7 +5999,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77088438"/>
+        <c:crossAx val="46670391"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6011,7 +6007,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77088438"/>
+        <c:axId val="46670391"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -6089,7 +6085,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53738799"/>
+        <c:crossAx val="43587432"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -6618,11 +6614,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="17587937"/>
-        <c:axId val="52720770"/>
+        <c:axId val="82480801"/>
+        <c:axId val="41558464"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="17587937"/>
+        <c:axId val="82480801"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6654,7 +6650,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52720770"/>
+        <c:crossAx val="41558464"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6662,7 +6658,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52720770"/>
+        <c:axId val="41558464"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -6740,7 +6736,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17587937"/>
+        <c:crossAx val="82480801"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -7269,11 +7265,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="73983087"/>
-        <c:axId val="94289784"/>
+        <c:axId val="4631275"/>
+        <c:axId val="70842767"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="73983087"/>
+        <c:axId val="4631275"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7305,7 +7301,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94289784"/>
+        <c:crossAx val="70842767"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7313,7 +7309,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94289784"/>
+        <c:axId val="70842767"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -7391,7 +7387,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73983087"/>
+        <c:crossAx val="4631275"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -7470,7 +7466,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>고3 모의고사·수능 · 총점</a:t>
+              <a:t>고3 모의고사 · 총점</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -7493,7 +7489,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A6</c:f>
+              <c:f>'고3 모의고사'!A6</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7549,7 +7545,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:f>'고3 모의고사'!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7561,7 +7557,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$6</c:f>
+              <c:f>'고3 모의고사'!$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -7578,7 +7574,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A7</c:f>
+              <c:f>'고3 모의고사'!A7</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7634,7 +7630,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:f>'고3 모의고사'!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7646,7 +7642,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$7</c:f>
+              <c:f>'고3 모의고사'!$B$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -7663,7 +7659,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A8</c:f>
+              <c:f>'고3 모의고사'!A8</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7719,7 +7715,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:f>'고3 모의고사'!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7731,7 +7727,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$8</c:f>
+              <c:f>'고3 모의고사'!$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -7748,7 +7744,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A9</c:f>
+              <c:f>'고3 모의고사'!A9</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7804,7 +7800,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$5</c:f>
+              <c:f>'고3 모의고사'!$B$5</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7816,7 +7812,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$9</c:f>
+              <c:f>'고3 모의고사'!$B$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -7836,11 +7832,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="84048133"/>
-        <c:axId val="52934726"/>
+        <c:axId val="27328697"/>
+        <c:axId val="14200844"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="84048133"/>
+        <c:axId val="27328697"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7872,7 +7868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52934726"/>
+        <c:crossAx val="14200844"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7880,7 +7876,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52934726"/>
+        <c:axId val="14200844"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -7958,7 +7954,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84048133"/>
+        <c:crossAx val="27328697"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -8037,7 +8033,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>고3 모의고사·수능 · 듣기</a:t>
+              <a:t>고3 모의고사 · 듣기</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -8060,7 +8056,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A14</c:f>
+              <c:f>'고3 모의고사'!A14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8116,7 +8112,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:f>'고3 모의고사'!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8128,7 +8124,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$14</c:f>
+              <c:f>'고3 모의고사'!$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8145,7 +8141,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A15</c:f>
+              <c:f>'고3 모의고사'!A15</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8201,7 +8197,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:f>'고3 모의고사'!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8213,7 +8209,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$15</c:f>
+              <c:f>'고3 모의고사'!$B$15</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8230,7 +8226,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A16</c:f>
+              <c:f>'고3 모의고사'!A16</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8286,7 +8282,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:f>'고3 모의고사'!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8298,7 +8294,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$16</c:f>
+              <c:f>'고3 모의고사'!$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8315,7 +8311,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A17</c:f>
+              <c:f>'고3 모의고사'!A17</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8371,7 +8367,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$13</c:f>
+              <c:f>'고3 모의고사'!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8383,7 +8379,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$17</c:f>
+              <c:f>'고3 모의고사'!$B$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8403,11 +8399,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="16593772"/>
-        <c:axId val="48756552"/>
+        <c:axId val="78202092"/>
+        <c:axId val="60748171"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="16593772"/>
+        <c:axId val="78202092"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8439,7 +8435,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48756552"/>
+        <c:crossAx val="60748171"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8447,7 +8443,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48756552"/>
+        <c:axId val="60748171"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -8525,7 +8521,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16593772"/>
+        <c:crossAx val="78202092"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -8604,7 +8600,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>고3 모의고사·수능 · 독해</a:t>
+              <a:t>고3 모의고사 · 독해</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -8627,7 +8623,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A22</c:f>
+              <c:f>'고3 모의고사'!A22</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8683,7 +8679,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:f>'고3 모의고사'!$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8695,7 +8691,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$22</c:f>
+              <c:f>'고3 모의고사'!$B$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8712,7 +8708,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A23</c:f>
+              <c:f>'고3 모의고사'!A23</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8768,7 +8764,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:f>'고3 모의고사'!$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8780,7 +8776,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$23</c:f>
+              <c:f>'고3 모의고사'!$B$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8797,7 +8793,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A24</c:f>
+              <c:f>'고3 모의고사'!A24</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8853,7 +8849,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:f>'고3 모의고사'!$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8865,7 +8861,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$24</c:f>
+              <c:f>'고3 모의고사'!$B$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8882,7 +8878,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!A25</c:f>
+              <c:f>'고3 모의고사'!A25</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8938,7 +8934,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'고3 모의고사_수능'!$B$21</c:f>
+              <c:f>'고3 모의고사'!$B$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -8950,7 +8946,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'고3 모의고사_수능'!$B$25</c:f>
+              <c:f>'고3 모의고사'!$B$25</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
@@ -8970,11 +8966,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="28008604"/>
-        <c:axId val="77983308"/>
+        <c:axId val="43511266"/>
+        <c:axId val="93960023"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="28008604"/>
+        <c:axId val="43511266"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9006,7 +9002,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77983308"/>
+        <c:crossAx val="93960023"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9014,7 +9010,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77983308"/>
+        <c:axId val="93960023"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -9092,7 +9088,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28008604"/>
+        <c:crossAx val="43511266"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -9876,11 +9872,11 @@
         <v>22</v>
       </c>
       <c r="C11" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!C10</f>
+        <f aca="false">'고3 모의고사'!C10</f>
         <v>92.25</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!D10</f>
+        <f aca="false">'고3 모의고사'!D10</f>
         <v>92.25</v>
       </c>
       <c r="E11" s="9" t="n">
@@ -9896,11 +9892,11 @@
         <v>23</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!C18</f>
+        <f aca="false">'고3 모의고사'!C18</f>
         <v>17</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!D18</f>
+        <f aca="false">'고3 모의고사'!D18</f>
         <v>17</v>
       </c>
       <c r="E12" s="9" t="n">
@@ -9916,11 +9912,11 @@
         <v>24</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!C26</f>
+        <f aca="false">'고3 모의고사'!C26</f>
         <v>24.75</v>
       </c>
       <c r="D13" s="8" t="n">
-        <f aca="false">'고3 모의고사_수능'!D26</f>
+        <f aca="false">'고3 모의고사'!D26</f>
         <v>24.75</v>
       </c>
       <c r="E13" s="9" t="n">

</xml_diff>

<commit_message>
Correct 구성관 middle-3 2nd mock exam total to 93
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015bh4sYU41PMoBKwVo8YRab
</commit_message>
<xml_diff>
--- a/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
+++ b/output/isabel-cohorts/구성관반_시험수준별_성적.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="55">
   <si>
     <r>
       <rPr>
@@ -1029,153 +1029,6 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">이라 비교에서 제외했습니다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">· </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">중</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">차 구성관 총점은 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2025</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">년 성적표 두 장에 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">92</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">점과 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">93</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">점으로 다르게 적혀 있어</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">듣기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">독해 개수가 함께 적힌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">92</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">점을 사용했습니다</t>
     </r>
     <r>
       <rPr>
@@ -3842,11 +3695,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="16752297"/>
-        <c:axId val="73426723"/>
+        <c:axId val="88888648"/>
+        <c:axId val="52373411"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="16752297"/>
+        <c:axId val="88888648"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3878,7 +3731,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73426723"/>
+        <c:crossAx val="52373411"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3886,7 +3739,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="73426723"/>
+        <c:axId val="52373411"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -3964,7 +3817,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16752297"/>
+        <c:crossAx val="88888648"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -4577,11 +4430,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="10296452"/>
-        <c:axId val="13529544"/>
+        <c:axId val="5704138"/>
+        <c:axId val="9443073"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10296452"/>
+        <c:axId val="5704138"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4613,7 +4466,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13529544"/>
+        <c:crossAx val="9443073"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4621,7 +4474,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13529544"/>
+        <c:axId val="9443073"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -4699,7 +4552,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10296452"/>
+        <c:crossAx val="5704138"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -5312,11 +5165,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="38405688"/>
-        <c:axId val="69754615"/>
+        <c:axId val="22490526"/>
+        <c:axId val="95637114"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="38405688"/>
+        <c:axId val="22490526"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5348,7 +5201,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69754615"/>
+        <c:crossAx val="95637114"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5356,7 +5209,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69754615"/>
+        <c:axId val="95637114"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -5434,7 +5287,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="38405688"/>
+        <c:crossAx val="22490526"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -5630,7 +5483,7 @@
                   <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>92</c:v>
+                  <c:v>93</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5963,11 +5816,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="43587432"/>
-        <c:axId val="46670391"/>
+        <c:axId val="89985456"/>
+        <c:axId val="83103646"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43587432"/>
+        <c:axId val="89985456"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5999,7 +5852,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46670391"/>
+        <c:crossAx val="83103646"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6007,7 +5860,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46670391"/>
+        <c:axId val="83103646"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -6085,7 +5938,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43587432"/>
+        <c:crossAx val="89985456"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -6614,11 +6467,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="82480801"/>
-        <c:axId val="41558464"/>
+        <c:axId val="94242852"/>
+        <c:axId val="21786972"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="82480801"/>
+        <c:axId val="94242852"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6650,7 +6503,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41558464"/>
+        <c:crossAx val="21786972"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6658,7 +6511,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41558464"/>
+        <c:axId val="21786972"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -6736,7 +6589,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82480801"/>
+        <c:crossAx val="94242852"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -7265,11 +7118,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="4631275"/>
-        <c:axId val="70842767"/>
+        <c:axId val="35593452"/>
+        <c:axId val="37707505"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="4631275"/>
+        <c:axId val="35593452"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7301,7 +7154,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70842767"/>
+        <c:crossAx val="37707505"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7309,7 +7162,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="70842767"/>
+        <c:axId val="37707505"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -7387,7 +7240,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="4631275"/>
+        <c:crossAx val="35593452"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -7832,11 +7685,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="27328697"/>
-        <c:axId val="14200844"/>
+        <c:axId val="5895008"/>
+        <c:axId val="94955980"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="27328697"/>
+        <c:axId val="5895008"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7868,7 +7721,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14200844"/>
+        <c:crossAx val="94955980"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7876,7 +7729,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="14200844"/>
+        <c:axId val="94955980"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="100"/>
@@ -7954,7 +7807,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="27328697"/>
+        <c:crossAx val="5895008"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="10"/>
@@ -8399,11 +8252,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="78202092"/>
-        <c:axId val="60748171"/>
+        <c:axId val="96091086"/>
+        <c:axId val="58075662"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78202092"/>
+        <c:axId val="96091086"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8435,7 +8288,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60748171"/>
+        <c:crossAx val="58075662"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8443,7 +8296,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60748171"/>
+        <c:axId val="58075662"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="17"/>
@@ -8521,7 +8374,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78202092"/>
+        <c:crossAx val="96091086"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="1"/>
@@ -8966,11 +8819,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="43511266"/>
-        <c:axId val="93960023"/>
+        <c:axId val="57656181"/>
+        <c:axId val="56627113"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43511266"/>
+        <c:axId val="57656181"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9002,7 +8855,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93960023"/>
+        <c:crossAx val="56627113"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9010,7 +8863,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="93960023"/>
+        <c:axId val="56627113"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="28"/>
@@ -9088,7 +8941,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43511266"/>
+        <c:crossAx val="57656181"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="2"/>
@@ -9606,7 +9459,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -9684,11 +9537,6 @@
     <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -9719,37 +9567,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>21</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>22</v>
       </c>
       <c r="C5" s="8" t="n">
         <f aca="false">'고1 모의고사'!I10</f>
@@ -9766,10 +9614,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">'고1 모의고사'!I18</f>
@@ -9786,10 +9634,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">'고1 모의고사'!I26</f>
@@ -9806,10 +9654,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8" s="8" t="n">
         <f aca="false">'고2 모의고사'!F10</f>
@@ -9817,19 +9665,19 @@
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">'고2 모의고사'!G10</f>
-        <v>86.5</v>
+        <v>86.75</v>
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">D8-C8</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="8" t="n">
         <f aca="false">'고2 모의고사'!F18</f>
@@ -9846,10 +9694,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="8" t="n">
         <f aca="false">'고2 모의고사'!F26</f>
@@ -9866,10 +9714,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="8" t="n">
         <f aca="false">'고3 모의고사'!C10</f>
@@ -9886,10 +9734,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">'고3 모의고사'!C18</f>
@@ -9906,10 +9754,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" s="8" t="n">
         <f aca="false">'고3 모의고사'!C26</f>
@@ -9949,57 +9797,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="I5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="J5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="K5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>71</v>
@@ -10037,7 +9885,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>58</v>
@@ -10075,7 +9923,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>70</v>
@@ -10113,7 +9961,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>69</v>
@@ -10151,7 +9999,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
@@ -10196,47 +10044,47 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J13" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="K13" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>17</v>
@@ -10274,7 +10122,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>15</v>
@@ -10312,7 +10160,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>16</v>
@@ -10350,7 +10198,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>17</v>
@@ -10388,7 +10236,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
@@ -10433,47 +10281,47 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="G21" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="G21" s="5" t="s">
+      <c r="H21" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="I21" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="J21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="J21" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="K21" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B22" s="10" t="n">
         <v>16</v>
@@ -10511,7 +10359,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>12</v>
@@ -10549,7 +10397,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>16</v>
@@ -10587,7 +10435,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>15</v>
@@ -10625,7 +10473,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>
@@ -10694,48 +10542,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="F5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="H5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>89</v>
@@ -10747,7 +10595,7 @@
         <v>95</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">B6</f>
@@ -10755,16 +10603,16 @@
       </c>
       <c r="G6" s="7" t="n">
         <f aca="false">LOOKUP(9.99E+307,B6:E6)</f>
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H6" s="11" t="n">
         <f aca="false">G6-F6</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>92</v>
@@ -10793,7 +10641,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>94</v>
@@ -10822,7 +10670,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>69</v>
@@ -10851,7 +10699,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
@@ -10867,7 +10715,7 @@
       </c>
       <c r="E10" s="13" t="n">
         <f aca="false">IF(COUNT(E6:E9)=0,"",AVERAGE(E6:E9))</f>
-        <v>86.5</v>
+        <v>86.75</v>
       </c>
       <c r="F10" s="13" t="n">
         <f aca="false">B10</f>
@@ -10875,47 +10723,47 @@
       </c>
       <c r="G10" s="13" t="n">
         <f aca="false">LOOKUP(9.99E+307,B10:E10)</f>
-        <v>86.5</v>
+        <v>86.75</v>
       </c>
       <c r="H10" s="14" t="n">
         <f aca="false">G10-F10</f>
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="F13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="H13" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>16</v>
@@ -10944,7 +10792,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>17</v>
@@ -10973,7 +10821,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>17</v>
@@ -11002,7 +10850,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>16</v>
@@ -11031,7 +10879,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
@@ -11064,38 +10912,38 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="5" t="s">
-        <v>52</v>
-      </c>
       <c r="F21" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G21" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="H21" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B22" s="10" t="n">
         <v>25</v>
@@ -11124,7 +10972,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>25</v>
@@ -11153,7 +11001,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>26</v>
@@ -11182,7 +11030,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>17</v>
@@ -11211,7 +11059,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>
@@ -11268,39 +11116,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="E5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>100</v>
@@ -11320,7 +11168,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>100</v>
@@ -11340,7 +11188,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>87</v>
@@ -11360,7 +11208,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>82</v>
@@ -11380,7 +11228,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">IF(COUNT(B6:B9)=0,"",AVERAGE(B6:B9))</f>
@@ -11401,29 +11249,29 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>17</v>
@@ -11443,7 +11291,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>17</v>
@@ -11463,7 +11311,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>17</v>
@@ -11483,7 +11331,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>17</v>
@@ -11503,7 +11351,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">IF(COUNT(B14:B17)=0,"",AVERAGE(B14:B17))</f>
@@ -11524,29 +11372,29 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="E21" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B22" s="10" t="n">
         <v>28</v>
@@ -11566,7 +11414,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>28</v>
@@ -11586,7 +11434,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>23</v>
@@ -11606,7 +11454,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>20</v>
@@ -11626,7 +11474,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">IF(COUNT(B22:B25)=0,"",AVERAGE(B22:B25))</f>

</xml_diff>